<commit_message>
Expand seed list to 35 companies and add CSV export
- Add 7 verified companies: SDE Media, Mobile Billboard Miami (both serve
  Palm Beach), Bill Salter Outdoor, Idon Media, Blip Billboards, Intersection,
  View Outdoor. Now 35 companies, 17 serving Palm Beach.
- Add CSV export: write_csv() in excel.py + --csv flag on the CLI (bare flag
  writes alongside the .xlsx, or pass an explicit path).
- Regenerate data/florida_billboard_companies.xlsx and add matching .csv.
- Update README counts, flag table, and layout.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169X7FqU7js4G1ZKY5WjVsV
</commit_message>
<xml_diff>
--- a/florida-billboard-scraper/data/florida_billboard_companies.xlsx
+++ b/florida-billboard-scraper/data/florida_billboard_companies.xlsx
@@ -12,7 +12,7 @@
     <sheet name="About" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FL Billboard Companies'!$A$4:$Q$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FL Billboard Companies'!$A$4:$Q$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -511,7 +511,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>28 companies · Palm Beach County first · prices are quote-only (see Pricing Reference tab)</t>
+          <t>35 companies · Palm Beach County first · prices are quote-only (see Pricing Reference tab)</t>
         </is>
       </c>
     </row>
@@ -1406,22 +1406,22 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>DAT Media FL</t>
+          <t>Blip Billboards</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>West Palm Beach; South Florida</t>
+          <t>Statewide FL (self-serve digital)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Palm Beach; Broward; Miami-Dade</t>
+          <t>Statewide</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1441,7 +1441,7 @@
       <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>https://datmediafl.com/west-palm-beach-mobile-led-billboard-advertising/</t>
+          <t>https://www.blipbillboards.com/billboard-locations/florida/</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
@@ -1451,17 +1451,17 @@
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>Mobile LED truck; typically day/week rate — quote only</t>
+          <t>Self-serve digital; pay-per-play, any budget — dynamic pricing</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>Mobile digital LED billboard trucks.</t>
+          <t>Self-serve digital billboard marketplace; no minimum contract.</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
-          <t>datmediafl.com; WebSearch 2026-07-08</t>
+          <t>blipbillboards.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q16" s="4" t="inlineStr">
@@ -1473,22 +1473,22 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Fliphound</t>
+          <t>DAT Media FL</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Broker / agency / marketplace</t>
+          <t>Mobile / LED-truck operator</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>West Palm Beach; statewide (digital platform)</t>
+          <t>West Palm Beach; South Florida</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Palm Beach (+ statewide)</t>
+          <t>Palm Beach; Broward; Miami-Dade</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1508,7 +1508,7 @@
       <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>https://fliphound.com/billboard-advertising/Florida/West-Palm-Beach</t>
+          <t>https://datmediafl.com/west-palm-beach-mobile-led-billboard-advertising/</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
@@ -1518,17 +1518,17 @@
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>Self-serve digital billboard booking — dynamic pricing</t>
+          <t>Mobile LED truck; typically day/week rate — quote only</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>Online marketplace/platform for digital billboards.</t>
+          <t>Mobile digital LED billboard trucks.</t>
         </is>
       </c>
       <c r="P17" s="4" t="inlineStr">
         <is>
-          <t>fliphound.com; WebSearch 2026-07-08</t>
+          <t>datmediafl.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q17" s="4" t="inlineStr">
@@ -1540,22 +1540,22 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Hanging Pants Media</t>
+          <t>Fliphound</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Miami; Ft. Lauderdale; WPB; Tampa; Orlando; Jacksonville</t>
+          <t>West Palm Beach; statewide (digital platform)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Statewide (major metros)</t>
+          <t>Palm Beach (+ statewide)</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -1575,7 +1575,7 @@
       <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>https://hangingpantsmedia.com/</t>
+          <t>https://fliphound.com/billboard-advertising/Florida/West-Palm-Beach</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
@@ -1585,17 +1585,17 @@
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>Static ~$800–$15k/mo; digital ~$1.2k–$25k+/mo (FL market avg)</t>
+          <t>Self-serve digital billboard booking — dynamic pricing</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>Works across all major FL markets incl. West Palm Beach.</t>
+          <t>Online marketplace/platform for digital billboards.</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>hangingpantsmedia.com; WebSearch 2026-07-08</t>
+          <t>fliphound.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q18" s="4" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Media Lease OOH</t>
+          <t>Hanging Pants Media</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1617,12 +1617,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>West Palm Beach; Fort Pierce</t>
+          <t>Miami; Ft. Lauderdale; WPB; Tampa; Orlando; Jacksonville</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Palm Beach; St. Lucie</t>
+          <t>Statewide (major metros)</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1642,172 +1642,176 @@
       <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="4" t="inlineStr">
         <is>
+          <t>https://hangingpantsmedia.com/</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>Static ~$800–$15k/mo; digital ~$1.2k–$25k+/mo (FL market avg)</t>
+        </is>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Geo-targets Palm Beach/Broward/Miami-Dade incl. Boca Raton, Delray, Palm Beach; I-95, I-595, Turnpike, US-1 inventory.</t>
+        </is>
+      </c>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>hangingpantsmedia.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Media Lease OOH</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Regional operator</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>West Palm Beach; Fort Pierce</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Palm Beach; St. Lucie</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
           <t>https://www.medialeaseooh.com/west-palm-beach-ft-pierce-fl/</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
-        <is>
-          <t>Quote only — request from company</t>
-        </is>
-      </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>Static ~$800–$15k/mo; digital ~$1.2k–$25k+/mo (FL market avg)</t>
         </is>
       </c>
-      <c r="O19" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>Out-of-home billboard leasing, WPB &amp; Ft. Pierce corridor.</t>
         </is>
       </c>
-      <c r="P19" s="4" t="inlineStr">
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>medialeaseooh.com; WebSearch 2026-07-08</t>
         </is>
       </c>
-      <c r="Q19" s="4" t="inlineStr">
+      <c r="Q20" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Clear Channel Outdoor — Miami</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>National operator</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Miami-Dade</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Miami-Dade; Broward</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>5800 NW 77th Court</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Miami</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Mobile Billboard Miami</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Miami; Broward; Palm Beach</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Miami-Dade; Broward; Palm Beach</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>6011 Rodman St, Unit 102</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Hollywood</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>33166</t>
-        </is>
-      </c>
-      <c r="J20" s="5" t="inlineStr"/>
-      <c r="K20" s="5" t="inlineStr"/>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>https://clearchanneloutdoor.com/</t>
-        </is>
-      </c>
-      <c r="M20" s="5" t="inlineStr">
-        <is>
-          <t>Quote only — request from company</t>
-        </is>
-      </c>
-      <c r="N20" s="5" t="inlineStr">
-        <is>
-          <t>Static ~$800–$15k/mo; digital ~$1.2k–$25k+/mo (FL market avg)</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr"/>
-      <c r="P20" s="5" t="inlineStr">
-        <is>
-          <t>WebSearch 2026-07-08</t>
-        </is>
-      </c>
-      <c r="Q20" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Carter Outdoor Advertising</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Regional operator</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>South Florida</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Broward; Miami-Dade; Palm Beach</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr"/>
-      <c r="G21" s="5" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="inlineStr"/>
-      <c r="K21" s="5" t="inlineStr"/>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>https://www.carteroutdoor.com/</t>
-        </is>
-      </c>
-      <c r="M21" s="5" t="inlineStr">
-        <is>
-          <t>Quote only — request from company</t>
-        </is>
-      </c>
-      <c r="N21" s="5" t="inlineStr">
-        <is>
-          <t>Static ~$800–$15k/mo; digital ~$1.2k–$25k+/mo (FL market avg)</t>
-        </is>
-      </c>
-      <c r="O21" s="5" t="inlineStr">
-        <is>
-          <t>Family-owned, serving South Florida since 1956.</t>
-        </is>
-      </c>
-      <c r="P21" s="5" t="inlineStr">
-        <is>
-          <t>carteroutdoor.com; WebSearch 2026-07-08</t>
-        </is>
-      </c>
-      <c r="Q21" s="5" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>33023</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mobilebillboardmiami.com/</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>Mobile LED truck — day/route rate, quote only</t>
+        </is>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>13+ yrs; digital LED billboard trucks, event marketing, live streaming.</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>mobilebillboardmiami.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q21" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1816,33 +1820,37 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Creative Outdoor Advertising</t>
+          <t>Clear Channel Outdoor — Miami</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Regional operator</t>
+          <t>National operator</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Tampa / Gulf Coast</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Hillsborough; Pinellas; Gulf Coast</t>
+          <t>Miami-Dade; Broward</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr"/>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>5800 NW 77th Court</t>
+        </is>
+      </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Tampa</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
@@ -1850,10 +1858,18 @@
           <t>FL</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr"/>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>33166</t>
+        </is>
+      </c>
       <c r="J22" s="5" t="inlineStr"/>
       <c r="K22" s="5" t="inlineStr"/>
-      <c r="L22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>https://clearchanneloutdoor.com/</t>
+        </is>
+      </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -1861,14 +1877,10 @@
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>Quote only</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr">
-        <is>
-          <t>HQ Tampa since 1984, 100+ employees, Florida Gulf Coast coverage.</t>
-        </is>
-      </c>
+          <t>Static ~$800–$15k/mo; digital ~$1.2k–$25k+/mo (FL market avg)</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr">
         <is>
           <t>WebSearch 2026-07-08</t>
@@ -1876,14 +1888,14 @@
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Logan Outdoor Advertising</t>
+          <t>Carter Outdoor Advertising</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1893,17 +1905,17 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Central West Florida</t>
+          <t>South Florida</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Six central FL counties</t>
+          <t>Broward; Miami-Dade; Palm Beach</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr"/>
@@ -1918,7 +1930,7 @@
       <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="5" t="inlineStr">
         <is>
-          <t>https://loganoutdoor.com/</t>
+          <t>https://www.carteroutdoor.com/</t>
         </is>
       </c>
       <c r="M23" s="5" t="inlineStr">
@@ -1928,13 +1940,17 @@
       </c>
       <c r="N23" s="5" t="inlineStr">
         <is>
-          <t>Quote only</t>
-        </is>
-      </c>
-      <c r="O23" s="5" t="inlineStr"/>
+          <t>Static ~$800–$15k/mo; digital ~$1.2k–$25k+/mo (FL market avg)</t>
+        </is>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>Family-owned, serving South Florida since 1956.</t>
+        </is>
+      </c>
       <c r="P23" s="5" t="inlineStr">
         <is>
-          <t>loganoutdoor.com; WebSearch 2026-07-08</t>
+          <t>carteroutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q23" s="5" t="inlineStr">
@@ -1946,7 +1962,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Orlando Outdoor Advertising</t>
+          <t>Creative Outdoor Advertising</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1956,12 +1972,12 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Orlando / Central Florida</t>
+          <t>Tampa / Gulf Coast</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Orange; Osceola; Seminole</t>
+          <t>Hillsborough; Pinellas; Gulf Coast</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1970,7 +1986,11 @@
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr"/>
-      <c r="G24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Tampa</t>
+        </is>
+      </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
           <t>FL</t>
@@ -1992,7 +2012,7 @@
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
-          <t>500+ faces across I-4 and theme-park routes.</t>
+          <t>HQ Tampa since 1984, 100+ employees, Florida Gulf Coast coverage.</t>
         </is>
       </c>
       <c r="P24" s="5" t="inlineStr">
@@ -2009,7 +2029,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Premium Outdoor</t>
+          <t>Logan Outdoor Advertising</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -2019,12 +2039,12 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Florida Panhandle</t>
+          <t>Central West Florida</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Escambia; Santa Rosa; Okaloosa; Bay (Panhandle)</t>
+          <t>Six central FL counties</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -2044,7 +2064,7 @@
       <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="5" t="inlineStr">
         <is>
-          <t>https://premiumoutdoor.com/</t>
+          <t>https://loganoutdoor.com/</t>
         </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
@@ -2057,14 +2077,10 @@
           <t>Quote only</t>
         </is>
       </c>
-      <c r="O25" s="5" t="inlineStr">
-        <is>
-          <t>Independently owned; 140+ digital &amp; static faces in the Panhandle.</t>
-        </is>
-      </c>
+      <c r="O25" s="5" t="inlineStr"/>
       <c r="P25" s="5" t="inlineStr">
         <is>
-          <t>premiumoutdoor.com; WebSearch 2026-07-08</t>
+          <t>loganoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q25" s="5" t="inlineStr">
@@ -2076,7 +2092,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>3N Outdoor Media</t>
+          <t>Orlando Outdoor Advertising</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -2086,17 +2102,17 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Miami</t>
+          <t>Orlando / Central Florida</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Miami-Dade</t>
+          <t>Orange; Osceola; Seminole</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr"/>
@@ -2115,10 +2131,14 @@
           <t>Quote only — request from company</t>
         </is>
       </c>
-      <c r="N26" s="5" t="inlineStr"/>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>Quote only</t>
+        </is>
+      </c>
       <c r="O26" s="5" t="inlineStr">
         <is>
-          <t>Miami-based; premium inventory along Biscayne Blvd and near airports.</t>
+          <t>500+ faces across I-4 and theme-park routes.</t>
         </is>
       </c>
       <c r="P26" s="5" t="inlineStr">
@@ -2128,34 +2148,34 @@
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Ilum Advertising</t>
+          <t>Premium Outdoor</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Orlando; Miami; Tampa; Jacksonville</t>
+          <t>Florida Panhandle</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Statewide (major metros)</t>
+          <t>Escambia; Santa Rosa; Okaloosa; Bay (Panhandle)</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr"/>
@@ -2168,7 +2188,11 @@
       <c r="I27" s="5" t="inlineStr"/>
       <c r="J27" s="5" t="inlineStr"/>
       <c r="K27" s="5" t="inlineStr"/>
-      <c r="L27" s="5" t="inlineStr"/>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>https://premiumoutdoor.com/</t>
+        </is>
+      </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -2176,25 +2200,29 @@
       </c>
       <c r="N27" s="5" t="inlineStr">
         <is>
-          <t>Mobile LED truck — day/week rate, quote only</t>
-        </is>
-      </c>
-      <c r="O27" s="5" t="inlineStr"/>
+          <t>Quote only</t>
+        </is>
+      </c>
+      <c r="O27" s="5" t="inlineStr">
+        <is>
+          <t>Independently owned; 140+ digital &amp; static faces in the Panhandle.</t>
+        </is>
+      </c>
       <c r="P27" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>premiumoutdoor.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q27" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Koala Outdoor Advertising</t>
+          <t>SDE Media</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -2204,25 +2232,21 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Polk County</t>
+          <t>Greater Miami</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Polk</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>Lake Hamilton</t>
-        </is>
-      </c>
+      <c r="G28" s="5" t="inlineStr"/>
       <c r="H28" s="5" t="inlineStr">
         <is>
           <t>FL</t>
@@ -2231,7 +2255,11 @@
       <c r="I28" s="5" t="inlineStr"/>
       <c r="J28" s="5" t="inlineStr"/>
       <c r="K28" s="5" t="inlineStr"/>
-      <c r="L28" s="5" t="inlineStr"/>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>https://sde-media.com/</t>
+        </is>
+      </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -2239,45 +2267,49 @@
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>Quote only</t>
-        </is>
-      </c>
-      <c r="O28" s="5" t="inlineStr"/>
+          <t>Static ~$800–$15k/mo; digital ~$1.2k–$25k+/mo (FL market avg)</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="inlineStr">
+        <is>
+          <t>Boutique independent; static + digital on Palmetto (SR 826), Dolphin (SR 836) &amp; Florida's Turnpike. FL Certified Minority Business; on Miami-Dade Asset Marketing Pool.</t>
+        </is>
+      </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>sde-media.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Lakeland Outdoor Advertising</t>
+          <t>3N Outdoor Media</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Lakeland / Central FL</t>
+          <t>Miami</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Hillsborough; Lake</t>
+          <t>Miami-Dade</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr"/>
@@ -2296,12 +2328,12 @@
           <t>Quote only — request from company</t>
         </is>
       </c>
-      <c r="N29" s="5" t="inlineStr">
-        <is>
-          <t>Quote only</t>
-        </is>
-      </c>
-      <c r="O29" s="5" t="inlineStr"/>
+      <c r="N29" s="5" t="inlineStr"/>
+      <c r="O29" s="5" t="inlineStr">
+        <is>
+          <t>Miami-based; premium inventory along Biscayne Blvd and near airports.</t>
+        </is>
+      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
           <t>WebSearch 2026-07-08</t>
@@ -2316,31 +2348,35 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Movia Media</t>
+          <t>Bill Salter Outdoor Advertising</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Mobile / LED-truck operator</t>
+          <t>Regional operator</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Florida (mobile)</t>
+          <t>Northwest Florida Panhandle</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Statewide</t>
+          <t>Escambia; Santa Rosa; Okaloosa (NW FL)</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Milton</t>
+        </is>
+      </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
           <t>FL</t>
@@ -2349,11 +2385,7 @@
       <c r="I30" s="5" t="inlineStr"/>
       <c r="J30" s="5" t="inlineStr"/>
       <c r="K30" s="5" t="inlineStr"/>
-      <c r="L30" s="5" t="inlineStr">
-        <is>
-          <t>https://moviamedia.com/</t>
-        </is>
-      </c>
+      <c r="L30" s="5" t="inlineStr"/>
       <c r="M30" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -2361,13 +2393,17 @@
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>Mobile billboard — quote only</t>
-        </is>
-      </c>
-      <c r="O30" s="5" t="inlineStr"/>
+          <t>Quote only</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>Long-standing regional independent operator in the western Panhandle.</t>
+        </is>
+      </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
-          <t>moviamedia.com; WebSearch 2026-07-08</t>
+          <t>WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
@@ -2379,27 +2415,27 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Smallwood Sign Company</t>
+          <t>Idon Media, LLC</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Independent / local operator</t>
+          <t>Broker / agency / marketplace</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Citrus / Orange counties</t>
+          <t>Florida (independent-operator network)</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Citrus; Orange</t>
+          <t>Statewide</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr"/>
@@ -2412,7 +2448,11 @@
       <c r="I31" s="5" t="inlineStr"/>
       <c r="J31" s="5" t="inlineStr"/>
       <c r="K31" s="5" t="inlineStr"/>
-      <c r="L31" s="5" t="inlineStr"/>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>http://www.idonmedia.com/about-us</t>
+        </is>
+      </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
           <t>Quote only — request from company</t>
@@ -2423,10 +2463,14 @@
           <t>Quote only</t>
         </is>
       </c>
-      <c r="O31" s="5" t="inlineStr"/>
+      <c r="O31" s="5" t="inlineStr">
+        <is>
+          <t>FL subsidiary of Digital Outdoor Advertising, LLC; represents independent billboard operators for national reach.</t>
+        </is>
+      </c>
       <c r="P31" s="5" t="inlineStr">
         <is>
-          <t>WebSearch 2026-07-08</t>
+          <t>idonmedia.com; WebSearch 2026-07-08</t>
         </is>
       </c>
       <c r="Q31" s="5" t="inlineStr">
@@ -2438,7 +2482,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>UMedia</t>
+          <t>Ilum Advertising</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -2448,7 +2492,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Miami; Orlando; Tampa; Daytona; Jacksonville</t>
+          <t>Orlando; Miami; Tampa; Jacksonville</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -2494,8 +2538,441 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Intersection</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>National operator</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>National transit / place-based (FL metros)</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Statewide FL (transit &amp; place-based)</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr"/>
+      <c r="J33" s="5" t="inlineStr"/>
+      <c r="K33" s="5" t="inlineStr"/>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>https://www.intersection.com/</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>Quote only</t>
+        </is>
+      </c>
+      <c r="O33" s="5" t="inlineStr">
+        <is>
+          <t>National OOH vendor; transit and place-based media, active in FL markets.</t>
+        </is>
+      </c>
+      <c r="P33" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Koala Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Polk County</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Polk</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Lake Hamilton</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr"/>
+      <c r="J34" s="5" t="inlineStr"/>
+      <c r="K34" s="5" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr"/>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>Quote only</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="inlineStr"/>
+      <c r="P34" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Lakeland Outdoor Advertising</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Lakeland / Central FL</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Hillsborough; Lake</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr"/>
+      <c r="J35" s="5" t="inlineStr"/>
+      <c r="K35" s="5" t="inlineStr"/>
+      <c r="L35" s="5" t="inlineStr"/>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>Quote only</t>
+        </is>
+      </c>
+      <c r="O35" s="5" t="inlineStr"/>
+      <c r="P35" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Movia Media</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Florida (mobile)</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Statewide</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr"/>
+      <c r="J36" s="5" t="inlineStr"/>
+      <c r="K36" s="5" t="inlineStr"/>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>https://moviamedia.com/</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>Mobile billboard — quote only</t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="inlineStr"/>
+      <c r="P36" s="5" t="inlineStr">
+        <is>
+          <t>moviamedia.com; WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Smallwood Sign Company</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Independent / local operator</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Citrus / Orange counties</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Citrus; Orange</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr"/>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr"/>
+      <c r="J37" s="5" t="inlineStr"/>
+      <c r="K37" s="5" t="inlineStr"/>
+      <c r="L37" s="5" t="inlineStr"/>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>Quote only</t>
+        </is>
+      </c>
+      <c r="O37" s="5" t="inlineStr"/>
+      <c r="P37" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>UMedia</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Mobile / LED-truck operator</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Miami; Orlando; Tampa; Daytona; Jacksonville</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Statewide (major metros)</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr"/>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr"/>
+      <c r="J38" s="5" t="inlineStr"/>
+      <c r="K38" s="5" t="inlineStr"/>
+      <c r="L38" s="5" t="inlineStr"/>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>Mobile LED truck — day/week rate, quote only</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr"/>
+      <c r="P38" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>View Outdoor</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>National operator</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Florida (OOH vendor)</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Statewide FL</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr"/>
+      <c r="G39" s="5" t="inlineStr"/>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr"/>
+      <c r="J39" s="5" t="inlineStr"/>
+      <c r="K39" s="5" t="inlineStr"/>
+      <c r="L39" s="5" t="inlineStr"/>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>Quote only — request from company</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>Quote only</t>
+        </is>
+      </c>
+      <c r="O39" s="5" t="inlineStr">
+        <is>
+          <t>Named among major OOH vendors operating in Florida.</t>
+        </is>
+      </c>
+      <c r="P39" s="5" t="inlineStr">
+        <is>
+          <t>WebSearch 2026-07-08</t>
+        </is>
+      </c>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:Q32"/>
+  <autoFilter ref="A4:Q39"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A1:Q1"/>
@@ -2761,7 +3238,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Generated by fbscraper v1.0 · 28 companies · scope: all Florida · sources: seed.</t>
+          <t>Generated by fbscraper v1.0 · 35 companies · scope: all Florida · sources: seed.</t>
         </is>
       </c>
     </row>

</xml_diff>